<commit_message>
Updated 0_Creating_GIN_Clusters to account for new plots
</commit_message>
<xml_diff>
--- a/Supplemental_Tables/Table_S5.xlsx
+++ b/Supplemental_Tables/Table_S5.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kierstenruff/Documents/Collaborations/Su/2024/IDR_Basis_Set/2025_02/Supplemental_Tables/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kierstenruff/Documents/GitHub/RUFF_KING_Grammars_of_IDRs_using_NARDINI-/Supplemental_Tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{563FE69D-E140-8447-A0DB-F9880B7D5874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C573F50-F6AE-8641-A6C8-4A405F85B3DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11640" yWindow="760" windowWidth="22920" windowHeight="16940" activeTab="10" xr2:uid="{9CB369E3-8528-1643-A6B4-7829535E3C5C}"/>
+    <workbookView xWindow="11080" yWindow="3160" windowWidth="22920" windowHeight="16940" firstSheet="4" activeTab="10" xr2:uid="{9CB369E3-8528-1643-A6B4-7829535E3C5C}"/>
   </bookViews>
   <sheets>
     <sheet name="Fig_5A" sheetId="9" r:id="rId1"/>
@@ -33,7 +33,10 @@
     <sheet name="Fig_S5B" sheetId="7" r:id="rId18"/>
     <sheet name="Fig_S5C" sheetId="8" r:id="rId19"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'top_80_pos-pos'!$A$1:$F$81</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -22256,6 +22259,7 @@
       <c r="F81" s="1"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F81" xr:uid="{5D340DDA-AF6D-B948-AF07-AFA02DBFF5A9}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>